<commit_message>
Update respiratory tracker through week of 10/5/2026
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BwtiE1oBBRcqVj5udzXLFk
</commit_message>
<xml_diff>
--- a/respiratory/RV_Tracker.xlsx
+++ b/respiratory/RV_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emilyjanoff/Desktop/MCPH/Reports/Resp Virus Reports/26-27/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33039559-486A-2243-920D-163B0E2DF733}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5F92BF8-8F20-6C4A-8318-E310E43E7FDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1480" yWindow="3620" windowWidth="29440" windowHeight="19780" tabRatio="500" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8140" yWindow="3040" windowWidth="29440" windowHeight="19780" tabRatio="500" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
     <sheet name="Flu_Age_Vax" sheetId="9" r:id="rId9"/>
     <sheet name="Highlights" sheetId="10" r:id="rId10"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -225,7 +225,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="136">
   <si>
     <t>Mono County Respiratory Virus Tracker</t>
   </si>
@@ -631,6 +631,9 @@
   <si>
     <t>Moderate</t>
   </si>
+  <si>
+    <t>California is experiencing an early increase in seasonal flu activity, with positive tests, emergency department visits, and hospitalizations exceeding levels seen during September and October in prior seasons. The Bay Area is reporting very high flu test positivity. COVID-19 continues to circulate, although activity is decreasing and illness is less severe than in previous seasons. Staying up to date on recommended respiratory virus immunizations remains important, and CDPH’s Respiratory Virus Hub provides information on prevention, vaccination, testing, and treatment.</t>
+  </si>
 </sst>
 </file>
 
@@ -640,7 +643,7 @@
     <numFmt numFmtId="164" formatCode="m/d/yyyy"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -698,6 +701,14 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -749,10 +760,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -780,8 +792,11 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1162,7 +1177,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1200,6 +1215,17 @@
         <v>127</v>
       </c>
       <c r="C3" s="6" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="18">
+        <v>46308</v>
+      </c>
+      <c r="B4" t="s">
+        <v>135</v>
+      </c>
+      <c r="C4" t="s">
         <v>128</v>
       </c>
     </row>
@@ -12917,26 +12943,47 @@
       <c r="A203" s="8">
         <v>46300</v>
       </c>
-      <c r="B203" s="6"/>
-      <c r="C203" s="6"/>
-      <c r="D203" s="6"/>
-      <c r="E203" s="6"/>
-      <c r="F203" s="6"/>
-      <c r="G203" s="6"/>
-      <c r="H203" s="6"/>
-      <c r="I203" s="6"/>
-      <c r="J203" s="6"/>
+      <c r="B203" s="6">
+        <v>1</v>
+      </c>
+      <c r="C203" s="6">
+        <v>0</v>
+      </c>
+      <c r="D203" s="6">
+        <v>0</v>
+      </c>
+      <c r="E203" s="6">
+        <v>0</v>
+      </c>
+      <c r="F203" s="6">
+        <v>0</v>
+      </c>
+      <c r="G203" s="6">
+        <v>2</v>
+      </c>
+      <c r="H203" s="6">
+        <v>0</v>
+      </c>
+      <c r="I203" s="6">
+        <v>0</v>
+      </c>
+      <c r="J203" s="6">
+        <v>0</v>
+      </c>
       <c r="K203" s="6"/>
       <c r="L203" s="6"/>
       <c r="M203" s="5" t="str">
         <f t="shared" si="18"/>
         <v/>
       </c>
-      <c r="N203" s="6"/>
-      <c r="O203" s="6"/>
-      <c r="P203" s="10" t="str">
-        <f t="shared" si="19"/>
-        <v/>
+      <c r="N203" s="6">
+        <v>0</v>
+      </c>
+      <c r="O203" s="6">
+        <v>2</v>
+      </c>
+      <c r="P203" s="10">
+        <v>0</v>
       </c>
       <c r="Q203" s="7"/>
       <c r="R203" s="11">
@@ -17176,23 +17223,35 @@
       <c r="A77" s="8">
         <v>46300</v>
       </c>
-      <c r="B77" s="6"/>
-      <c r="C77" s="6"/>
-      <c r="D77" s="10" t="str">
+      <c r="B77" s="6">
+        <v>1</v>
+      </c>
+      <c r="C77" s="6">
+        <v>6</v>
+      </c>
+      <c r="D77" s="10">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="E77" s="6"/>
-      <c r="F77" s="6"/>
-      <c r="G77" s="10" t="str">
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="E77" s="6">
+        <v>0</v>
+      </c>
+      <c r="F77" s="6">
+        <v>11</v>
+      </c>
+      <c r="G77" s="10">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="H77" s="6"/>
-      <c r="I77" s="6"/>
-      <c r="J77" s="10" t="str">
+        <v>0</v>
+      </c>
+      <c r="H77" s="6">
+        <v>0</v>
+      </c>
+      <c r="I77" s="6">
+        <v>11</v>
+      </c>
+      <c r="J77" s="10">
         <f t="shared" si="8"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K77" s="7"/>
     </row>
@@ -18196,9 +18255,9 @@
         <f>IF(COUNTIFS(Weekly_Local!$U:$U,"2025-26",Weekly_Local!$T:$T,$A9,Weekly_Local!$B:$B,"&lt;&gt;")=0,"",SUMIFS(Weekly_Local!$B:$B,Weekly_Local!$U:$U,"2025-26",Weekly_Local!$T:$T,$A9))</f>
         <v>2</v>
       </c>
-      <c r="F9" s="5" t="str">
+      <c r="F9" s="5">
         <f>IF(COUNTIFS(Weekly_Local!$U:$U,"2026-27",Weekly_Local!$T:$T,$A9,Weekly_Local!$B:$B,"&lt;&gt;")=0,"",SUMIFS(Weekly_Local!$B:$B,Weekly_Local!$U:$U,"2026-27",Weekly_Local!$T:$T,$A9))</f>
-        <v/>
+        <v>1</v>
       </c>
       <c r="G9" s="5" t="str">
         <f>IF(AND($A9=53,DATE(YEAR(Config!$B$3),1,4)-WEEKDAY(DATE(YEAR(Config!$B$3),1,4))+1+364&gt;=DATE(YEAR(Config!$B$3)+1,1,4)-WEEKDAY(DATE(YEAR(Config!$B$3)+1,1,4))+1),"",TEXT(DATE(YEAR(Config!$B$3)+IF($A9&gt;=36,0,1),1,4)-WEEKDAY(DATE(YEAR(Config!$B$3)+IF($A9&gt;=36,0,1),1,4))+1+7*($A9-1)+1,"m/d/yy")&amp;" – "&amp;TEXT(DATE(YEAR(Config!$B$3)+IF($A9&gt;=36,0,1),1,4)-WEEKDAY(DATE(YEAR(Config!$B$3)+IF($A9&gt;=36,0,1),1,4))+1+7*($A9-1)+7,"m/d/yy"))</f>
@@ -19760,9 +19819,9 @@
         <f>IF(COUNTIFS(Weekly_Local!$U:$U,"2025-26",Weekly_Local!$T:$T,$A66,Weekly_Local!$C:$C,"&lt;&gt;")=0,"",SUMIFS(Weekly_Local!$C:$C,Weekly_Local!$U:$U,"2025-26",Weekly_Local!$T:$T,$A66))</f>
         <v>0</v>
       </c>
-      <c r="F66" s="5" t="str">
+      <c r="F66" s="5">
         <f>IF(COUNTIFS(Weekly_Local!$U:$U,"2026-27",Weekly_Local!$T:$T,$A66,Weekly_Local!$C:$C,"&lt;&gt;")=0,"",SUMIFS(Weekly_Local!$C:$C,Weekly_Local!$U:$U,"2026-27",Weekly_Local!$T:$T,$A66))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G66" s="5" t="str">
         <f>IF(AND($A66=53,DATE(YEAR(Config!$B$3),1,4)-WEEKDAY(DATE(YEAR(Config!$B$3),1,4))+1+364&gt;=DATE(YEAR(Config!$B$3)+1,1,4)-WEEKDAY(DATE(YEAR(Config!$B$3)+1,1,4))+1),"",TEXT(DATE(YEAR(Config!$B$3)+IF($A66&gt;=36,0,1),1,4)-WEEKDAY(DATE(YEAR(Config!$B$3)+IF($A66&gt;=36,0,1),1,4))+1+7*($A66-1)+1,"m/d/yy")&amp;" – "&amp;TEXT(DATE(YEAR(Config!$B$3)+IF($A66&gt;=36,0,1),1,4)-WEEKDAY(DATE(YEAR(Config!$B$3)+IF($A66&gt;=36,0,1),1,4))+1+7*($A66-1)+7,"m/d/yy"))</f>
@@ -21324,9 +21383,9 @@
         <f>IF(COUNTIFS(Weekly_Local!$U:$U,"2025-26",Weekly_Local!$T:$T,$A123,Weekly_Local!$D:$D,"&lt;&gt;")=0,"",SUMIFS(Weekly_Local!$D:$D,Weekly_Local!$U:$U,"2025-26",Weekly_Local!$T:$T,$A123))</f>
         <v>0</v>
       </c>
-      <c r="F123" s="5" t="str">
+      <c r="F123" s="5">
         <f>IF(COUNTIFS(Weekly_Local!$U:$U,"2026-27",Weekly_Local!$T:$T,$A123,Weekly_Local!$D:$D,"&lt;&gt;")=0,"",SUMIFS(Weekly_Local!$D:$D,Weekly_Local!$U:$U,"2026-27",Weekly_Local!$T:$T,$A123))</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="G123" s="5" t="str">
         <f>IF(AND($A123=53,DATE(YEAR(Config!$B$3),1,4)-WEEKDAY(DATE(YEAR(Config!$B$3),1,4))+1+364&gt;=DATE(YEAR(Config!$B$3)+1,1,4)-WEEKDAY(DATE(YEAR(Config!$B$3)+1,1,4))+1),"",TEXT(DATE(YEAR(Config!$B$3)+IF($A123&gt;=36,0,1),1,4)-WEEKDAY(DATE(YEAR(Config!$B$3)+IF($A123&gt;=36,0,1),1,4))+1+7*($A123-1)+1,"m/d/yy")&amp;" – "&amp;TEXT(DATE(YEAR(Config!$B$3)+IF($A123&gt;=36,0,1),1,4)-WEEKDAY(DATE(YEAR(Config!$B$3)+IF($A123&gt;=36,0,1),1,4))+1+7*($A123-1)+7,"m/d/yy"))</f>
@@ -27495,9 +27554,7 @@
       <c r="E5" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="F5" s="6">
-        <v>0.95</v>
-      </c>
+      <c r="F5" s="6"/>
       <c r="G5" s="15"/>
       <c r="H5" s="15"/>
       <c r="I5" s="15"/>
@@ -27507,10 +27564,18 @@
       <c r="A6" s="8">
         <v>46300</v>
       </c>
-      <c r="B6" s="15"/>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="6"/>
+      <c r="B6" s="15">
+        <v>8.5999999999999993E-2</v>
+      </c>
+      <c r="C6" s="15">
+        <v>8.7999999999999995E-2</v>
+      </c>
+      <c r="D6" s="15">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>134</v>
+      </c>
       <c r="F6" s="6"/>
       <c r="G6" s="15"/>
       <c r="H6" s="15"/>
@@ -27994,7 +28059,7 @@
       <c r="J40" s="7"/>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
+      <c r="A44" s="17" t="s">
         <v>128</v>
       </c>
     </row>
@@ -28005,9 +28070,12 @@
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="A44" r:id="rId1" xr:uid="{0C5618FE-1065-7447-A4CF-86B455C694F8}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-  <legacyDrawing r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Tracker 10/13: Mammoth flu A/B for week of 10/5; highlights re-applied
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BwtiE1oBBRcqVj5udzXLFk
</commit_message>
<xml_diff>
--- a/respiratory/RV_Tracker.xlsx
+++ b/respiratory/RV_Tracker.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="9"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" state="visible" r:id="rId3"/>
@@ -622,7 +622,7 @@
     <t xml:space="preserve">Covid-19 test positivity in Mono County fell to 14% (1 of 7 tests), down from 31% the prior week. All 11 flu tests and all 11 RSV tests reported this week were negative.</t>
   </si>
   <si>
-    <t xml:space="preserve">Mammoth Hospital reported 2 flu patients this week, neither a Mono County resident. There were no Covid-19 or RSV patients. Local wastewater sampling has been paused since 9/9 and is expected to resume this week.</t>
+    <t xml:space="preserve">Mammoth Hospital reported 2 flu patients this week, both influenza A and neither a Mono County resident. There were no Covid-19 or RSV patients. Local wastewater sampling has been paused since 9/9 and is expected to resume this week.</t>
   </si>
   <si>
     <t xml:space="preserve">California is seeing an early rise in flu activity. Statewide flu test positivity reached 8.8%, up from 2.9% in early September. Positive tests, emergency department visits, and hospitalizations are above September–October levels in prior seasons, and the Bay Area is reporting very high flu test positivity. Covid-19 activity in California continues to decline, with statewide test positivity at 8.6%.</t>
@@ -13112,11 +13112,15 @@
       <c r="J203" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="K203" s="6"/>
-      <c r="L203" s="6"/>
-      <c r="M203" s="5" t="str">
+      <c r="K203" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="L203" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M203" s="5" t="n">
         <f aca="false">IF(AND(K203="",L203=""),"",SUM(K203:L203))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="N203" s="6" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Wastewater: measles-only chart and influenza A subtype (H1/H3/H5) chart
- Replace Verily other-targets chart (mpox no longer tested) with measles only
- New stacked bar chart of H1/H3/H5: share of subtype signal (low-signal weeks faded) or concentration
- Wastewater_Local gains H1, H3, Measles columns; parser reads columns by header
- Week of 10/19 entered for H1/H3/measles

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012tC3eUsd1X3X2aR7py7CH3
</commit_message>
<xml_diff>
--- a/respiratory/RV_Tracker.xlsx
+++ b/respiratory/RV_Tracker.xlsx
@@ -689,7 +689,7 @@
     <row r="7" ht="15" customHeight="1" s="20">
       <c r="A7" s="22" t="inlineStr">
         <is>
-          <t>3. Wastewater_Local: enter Verily values for the Mammoth plant and the current UC Davis trend table. These also feed the Cases vs wastewater tab.</t>
+          <t>3. Wastewater_Local: enter Verily values for the Mammoth plant (SARS-CoV-2, influenza A and B, RSV, H5, H1, H3, measles; weekly mean of virus ÷ PMMoV × 1,000,000) and the current UC Davis trend table. These also feed the Cases vs wastewater tab. Mpox is no longer tested under the new contract.</t>
         </is>
       </c>
     </row>
@@ -26782,13 +26782,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="19" min="1" max="4"/>
     <col width="10" customWidth="1" style="19" min="5" max="5"/>
     <col width="16" customWidth="1" style="19" min="6" max="6"/>
-    <col width="60" customWidth="1" style="19" min="7" max="7"/>
+    <col width="16" customWidth="1" style="19" min="7" max="7"/>
+    <col width="16" customWidth="1" style="20" min="8" max="8"/>
+    <col width="16" customWidth="1" style="20" min="9" max="9"/>
+    <col width="60" customWidth="1" style="20" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="31.5" customHeight="1" s="20">
@@ -26824,6 +26827,21 @@
       </c>
       <c r="G1" s="24" t="inlineStr">
         <is>
+          <t>Influenza A (H1)</t>
+        </is>
+      </c>
+      <c r="H1" s="24" t="inlineStr">
+        <is>
+          <t>Influenza A (H3)</t>
+        </is>
+      </c>
+      <c r="I1" s="24" t="inlineStr">
+        <is>
+          <t>Measles</t>
+        </is>
+      </c>
+      <c r="J1" s="24" t="inlineStr">
+        <is>
           <t>Notes</t>
         </is>
       </c>
@@ -26837,7 +26855,10 @@
       <c r="D2" s="26" t="n"/>
       <c r="E2" s="26" t="n"/>
       <c r="F2" s="26" t="n"/>
-      <c r="G2" s="27" t="n"/>
+      <c r="G2" s="26" t="n"/>
+      <c r="H2" s="26" t="n"/>
+      <c r="I2" s="26" t="n"/>
+      <c r="J2" s="27" t="n"/>
     </row>
     <row r="3" ht="15" customHeight="1" s="20">
       <c r="A3" s="28" t="n">
@@ -26848,7 +26869,10 @@
       <c r="D3" s="26" t="n"/>
       <c r="E3" s="26" t="n"/>
       <c r="F3" s="26" t="n"/>
-      <c r="G3" s="27" t="n"/>
+      <c r="G3" s="26" t="n"/>
+      <c r="H3" s="26" t="n"/>
+      <c r="I3" s="26" t="n"/>
+      <c r="J3" s="27" t="n"/>
     </row>
     <row r="4" ht="15" customHeight="1" s="20">
       <c r="A4" s="28" t="n">
@@ -26859,7 +26883,10 @@
       <c r="D4" s="26" t="n"/>
       <c r="E4" s="26" t="n"/>
       <c r="F4" s="26" t="n"/>
-      <c r="G4" s="27" t="n"/>
+      <c r="G4" s="26" t="n"/>
+      <c r="H4" s="26" t="n"/>
+      <c r="I4" s="26" t="n"/>
+      <c r="J4" s="27" t="n"/>
     </row>
     <row r="5" ht="15" customHeight="1" s="20">
       <c r="A5" s="28" t="n">
@@ -26870,7 +26897,10 @@
       <c r="D5" s="26" t="n"/>
       <c r="E5" s="26" t="n"/>
       <c r="F5" s="26" t="n"/>
-      <c r="G5" s="27" t="n"/>
+      <c r="G5" s="26" t="n"/>
+      <c r="H5" s="26" t="n"/>
+      <c r="I5" s="26" t="n"/>
+      <c r="J5" s="27" t="n"/>
     </row>
     <row r="6" ht="15" customHeight="1" s="20">
       <c r="A6" s="28" t="n">
@@ -26881,7 +26911,10 @@
       <c r="D6" s="26" t="n"/>
       <c r="E6" s="26" t="n"/>
       <c r="F6" s="26" t="n"/>
-      <c r="G6" s="27" t="n"/>
+      <c r="G6" s="26" t="n"/>
+      <c r="H6" s="26" t="n"/>
+      <c r="I6" s="26" t="n"/>
+      <c r="J6" s="27" t="n"/>
     </row>
     <row r="7" ht="15" customHeight="1" s="20">
       <c r="A7" s="28" t="n">
@@ -26892,7 +26925,10 @@
       <c r="D7" s="26" t="n"/>
       <c r="E7" s="26" t="n"/>
       <c r="F7" s="26" t="n"/>
-      <c r="G7" s="27" t="n"/>
+      <c r="G7" s="26" t="n"/>
+      <c r="H7" s="26" t="n"/>
+      <c r="I7" s="26" t="n"/>
+      <c r="J7" s="27" t="n"/>
     </row>
     <row r="8" ht="15" customHeight="1" s="20">
       <c r="A8" s="28" t="n">
@@ -26913,9 +26949,18 @@
       <c r="F8" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="27" t="inlineStr">
+      <c r="G8" s="26" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="H8" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="27" t="inlineStr">
         <is>
-          <t>1 sample (10/21), first under new contract. Influenza A H1 subtype detected at 4.02.</t>
+          <t>1 sample (10/21), first under new contract.</t>
         </is>
       </c>
     </row>
@@ -26928,7 +26973,10 @@
       <c r="D9" s="26" t="n"/>
       <c r="E9" s="26" t="n"/>
       <c r="F9" s="26" t="n"/>
-      <c r="G9" s="27" t="n"/>
+      <c r="G9" s="26" t="n"/>
+      <c r="H9" s="26" t="n"/>
+      <c r="I9" s="26" t="n"/>
+      <c r="J9" s="27" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1" s="20">
       <c r="A10" s="28" t="n">
@@ -26939,7 +26987,10 @@
       <c r="D10" s="26" t="n"/>
       <c r="E10" s="26" t="n"/>
       <c r="F10" s="26" t="n"/>
-      <c r="G10" s="27" t="n"/>
+      <c r="G10" s="26" t="n"/>
+      <c r="H10" s="26" t="n"/>
+      <c r="I10" s="26" t="n"/>
+      <c r="J10" s="27" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1" s="20">
       <c r="A11" s="28" t="n">
@@ -26950,7 +27001,10 @@
       <c r="D11" s="26" t="n"/>
       <c r="E11" s="26" t="n"/>
       <c r="F11" s="26" t="n"/>
-      <c r="G11" s="27" t="n"/>
+      <c r="G11" s="26" t="n"/>
+      <c r="H11" s="26" t="n"/>
+      <c r="I11" s="26" t="n"/>
+      <c r="J11" s="27" t="n"/>
     </row>
     <row r="12" ht="15" customHeight="1" s="20">
       <c r="A12" s="28" t="n">
@@ -26961,7 +27015,10 @@
       <c r="D12" s="26" t="n"/>
       <c r="E12" s="26" t="n"/>
       <c r="F12" s="26" t="n"/>
-      <c r="G12" s="27" t="n"/>
+      <c r="G12" s="26" t="n"/>
+      <c r="H12" s="26" t="n"/>
+      <c r="I12" s="26" t="n"/>
+      <c r="J12" s="27" t="n"/>
     </row>
     <row r="13" ht="15" customHeight="1" s="20">
       <c r="A13" s="28" t="n">
@@ -26972,7 +27029,10 @@
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
       <c r="F13" s="26" t="n"/>
-      <c r="G13" s="27" t="n"/>
+      <c r="G13" s="26" t="n"/>
+      <c r="H13" s="26" t="n"/>
+      <c r="I13" s="26" t="n"/>
+      <c r="J13" s="27" t="n"/>
     </row>
     <row r="14" ht="15" customHeight="1" s="20">
       <c r="A14" s="28" t="n">
@@ -26983,7 +27043,10 @@
       <c r="D14" s="26" t="n"/>
       <c r="E14" s="26" t="n"/>
       <c r="F14" s="26" t="n"/>
-      <c r="G14" s="27" t="n"/>
+      <c r="G14" s="26" t="n"/>
+      <c r="H14" s="26" t="n"/>
+      <c r="I14" s="26" t="n"/>
+      <c r="J14" s="27" t="n"/>
     </row>
     <row r="15" ht="15" customHeight="1" s="20">
       <c r="A15" s="28" t="n">
@@ -26994,7 +27057,10 @@
       <c r="D15" s="26" t="n"/>
       <c r="E15" s="26" t="n"/>
       <c r="F15" s="26" t="n"/>
-      <c r="G15" s="27" t="n"/>
+      <c r="G15" s="26" t="n"/>
+      <c r="H15" s="26" t="n"/>
+      <c r="I15" s="26" t="n"/>
+      <c r="J15" s="27" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1" s="20">
       <c r="A16" s="28" t="n">
@@ -27005,7 +27071,10 @@
       <c r="D16" s="26" t="n"/>
       <c r="E16" s="26" t="n"/>
       <c r="F16" s="26" t="n"/>
-      <c r="G16" s="27" t="n"/>
+      <c r="G16" s="26" t="n"/>
+      <c r="H16" s="26" t="n"/>
+      <c r="I16" s="26" t="n"/>
+      <c r="J16" s="27" t="n"/>
     </row>
     <row r="17" ht="15" customHeight="1" s="20">
       <c r="A17" s="28" t="n">
@@ -27016,7 +27085,10 @@
       <c r="D17" s="26" t="n"/>
       <c r="E17" s="26" t="n"/>
       <c r="F17" s="26" t="n"/>
-      <c r="G17" s="27" t="n"/>
+      <c r="G17" s="26" t="n"/>
+      <c r="H17" s="26" t="n"/>
+      <c r="I17" s="26" t="n"/>
+      <c r="J17" s="27" t="n"/>
     </row>
     <row r="18" ht="15" customHeight="1" s="20">
       <c r="A18" s="28" t="n">
@@ -27027,7 +27099,10 @@
       <c r="D18" s="26" t="n"/>
       <c r="E18" s="26" t="n"/>
       <c r="F18" s="26" t="n"/>
-      <c r="G18" s="27" t="n"/>
+      <c r="G18" s="26" t="n"/>
+      <c r="H18" s="26" t="n"/>
+      <c r="I18" s="26" t="n"/>
+      <c r="J18" s="27" t="n"/>
     </row>
     <row r="19" ht="15" customHeight="1" s="20">
       <c r="A19" s="28" t="n">
@@ -27038,7 +27113,10 @@
       <c r="D19" s="26" t="n"/>
       <c r="E19" s="26" t="n"/>
       <c r="F19" s="26" t="n"/>
-      <c r="G19" s="27" t="n"/>
+      <c r="G19" s="26" t="n"/>
+      <c r="H19" s="26" t="n"/>
+      <c r="I19" s="26" t="n"/>
+      <c r="J19" s="27" t="n"/>
     </row>
     <row r="20" ht="15" customHeight="1" s="20">
       <c r="A20" s="28" t="n">
@@ -27049,7 +27127,10 @@
       <c r="D20" s="26" t="n"/>
       <c r="E20" s="26" t="n"/>
       <c r="F20" s="26" t="n"/>
-      <c r="G20" s="27" t="n"/>
+      <c r="G20" s="26" t="n"/>
+      <c r="H20" s="26" t="n"/>
+      <c r="I20" s="26" t="n"/>
+      <c r="J20" s="27" t="n"/>
     </row>
     <row r="21" ht="15" customHeight="1" s="20">
       <c r="A21" s="28" t="n">
@@ -27060,7 +27141,10 @@
       <c r="D21" s="26" t="n"/>
       <c r="E21" s="26" t="n"/>
       <c r="F21" s="26" t="n"/>
-      <c r="G21" s="27" t="n"/>
+      <c r="G21" s="26" t="n"/>
+      <c r="H21" s="26" t="n"/>
+      <c r="I21" s="26" t="n"/>
+      <c r="J21" s="27" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1" s="20">
       <c r="A22" s="28" t="n">
@@ -27071,7 +27155,10 @@
       <c r="D22" s="26" t="n"/>
       <c r="E22" s="26" t="n"/>
       <c r="F22" s="26" t="n"/>
-      <c r="G22" s="27" t="n"/>
+      <c r="G22" s="26" t="n"/>
+      <c r="H22" s="26" t="n"/>
+      <c r="I22" s="26" t="n"/>
+      <c r="J22" s="27" t="n"/>
     </row>
     <row r="23" ht="15" customHeight="1" s="20">
       <c r="A23" s="28" t="n">
@@ -27082,7 +27169,10 @@
       <c r="D23" s="26" t="n"/>
       <c r="E23" s="26" t="n"/>
       <c r="F23" s="26" t="n"/>
-      <c r="G23" s="27" t="n"/>
+      <c r="G23" s="26" t="n"/>
+      <c r="H23" s="26" t="n"/>
+      <c r="I23" s="26" t="n"/>
+      <c r="J23" s="27" t="n"/>
     </row>
     <row r="24" ht="15" customHeight="1" s="20">
       <c r="A24" s="28" t="n">
@@ -27093,7 +27183,10 @@
       <c r="D24" s="26" t="n"/>
       <c r="E24" s="26" t="n"/>
       <c r="F24" s="26" t="n"/>
-      <c r="G24" s="27" t="n"/>
+      <c r="G24" s="26" t="n"/>
+      <c r="H24" s="26" t="n"/>
+      <c r="I24" s="26" t="n"/>
+      <c r="J24" s="27" t="n"/>
     </row>
     <row r="25" ht="15" customHeight="1" s="20">
       <c r="A25" s="28" t="n">
@@ -27104,7 +27197,10 @@
       <c r="D25" s="26" t="n"/>
       <c r="E25" s="26" t="n"/>
       <c r="F25" s="26" t="n"/>
-      <c r="G25" s="27" t="n"/>
+      <c r="G25" s="26" t="n"/>
+      <c r="H25" s="26" t="n"/>
+      <c r="I25" s="26" t="n"/>
+      <c r="J25" s="27" t="n"/>
     </row>
     <row r="26" ht="15" customHeight="1" s="20">
       <c r="A26" s="28" t="n">
@@ -27115,7 +27211,10 @@
       <c r="D26" s="26" t="n"/>
       <c r="E26" s="26" t="n"/>
       <c r="F26" s="26" t="n"/>
-      <c r="G26" s="27" t="n"/>
+      <c r="G26" s="26" t="n"/>
+      <c r="H26" s="26" t="n"/>
+      <c r="I26" s="26" t="n"/>
+      <c r="J26" s="27" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1" s="20">
       <c r="A27" s="28" t="n">
@@ -27126,7 +27225,10 @@
       <c r="D27" s="26" t="n"/>
       <c r="E27" s="26" t="n"/>
       <c r="F27" s="26" t="n"/>
-      <c r="G27" s="27" t="n"/>
+      <c r="G27" s="26" t="n"/>
+      <c r="H27" s="26" t="n"/>
+      <c r="I27" s="26" t="n"/>
+      <c r="J27" s="27" t="n"/>
     </row>
     <row r="28" ht="15" customHeight="1" s="20">
       <c r="A28" s="28" t="n">
@@ -27137,7 +27239,10 @@
       <c r="D28" s="26" t="n"/>
       <c r="E28" s="26" t="n"/>
       <c r="F28" s="26" t="n"/>
-      <c r="G28" s="27" t="n"/>
+      <c r="G28" s="26" t="n"/>
+      <c r="H28" s="26" t="n"/>
+      <c r="I28" s="26" t="n"/>
+      <c r="J28" s="27" t="n"/>
     </row>
     <row r="29" ht="15" customHeight="1" s="20">
       <c r="A29" s="28" t="n">
@@ -27148,7 +27253,10 @@
       <c r="D29" s="26" t="n"/>
       <c r="E29" s="26" t="n"/>
       <c r="F29" s="26" t="n"/>
-      <c r="G29" s="27" t="n"/>
+      <c r="G29" s="26" t="n"/>
+      <c r="H29" s="26" t="n"/>
+      <c r="I29" s="26" t="n"/>
+      <c r="J29" s="27" t="n"/>
     </row>
     <row r="30" ht="15" customHeight="1" s="20">
       <c r="A30" s="28" t="n">
@@ -27159,7 +27267,10 @@
       <c r="D30" s="26" t="n"/>
       <c r="E30" s="26" t="n"/>
       <c r="F30" s="26" t="n"/>
-      <c r="G30" s="27" t="n"/>
+      <c r="G30" s="26" t="n"/>
+      <c r="H30" s="26" t="n"/>
+      <c r="I30" s="26" t="n"/>
+      <c r="J30" s="27" t="n"/>
     </row>
     <row r="31" ht="15" customHeight="1" s="20">
       <c r="A31" s="28" t="n">
@@ -27170,7 +27281,10 @@
       <c r="D31" s="26" t="n"/>
       <c r="E31" s="26" t="n"/>
       <c r="F31" s="26" t="n"/>
-      <c r="G31" s="27" t="n"/>
+      <c r="G31" s="26" t="n"/>
+      <c r="H31" s="26" t="n"/>
+      <c r="I31" s="26" t="n"/>
+      <c r="J31" s="27" t="n"/>
     </row>
     <row r="32" ht="15" customHeight="1" s="20">
       <c r="A32" s="28" t="n">
@@ -27181,7 +27295,10 @@
       <c r="D32" s="26" t="n"/>
       <c r="E32" s="26" t="n"/>
       <c r="F32" s="26" t="n"/>
-      <c r="G32" s="27" t="n"/>
+      <c r="G32" s="26" t="n"/>
+      <c r="H32" s="26" t="n"/>
+      <c r="I32" s="26" t="n"/>
+      <c r="J32" s="27" t="n"/>
     </row>
     <row r="33" ht="15" customHeight="1" s="20">
       <c r="A33" s="28" t="n">
@@ -27192,7 +27309,10 @@
       <c r="D33" s="26" t="n"/>
       <c r="E33" s="26" t="n"/>
       <c r="F33" s="26" t="n"/>
-      <c r="G33" s="27" t="n"/>
+      <c r="G33" s="26" t="n"/>
+      <c r="H33" s="26" t="n"/>
+      <c r="I33" s="26" t="n"/>
+      <c r="J33" s="27" t="n"/>
     </row>
     <row r="34" ht="15" customHeight="1" s="20">
       <c r="A34" s="28" t="n">
@@ -27203,7 +27323,10 @@
       <c r="D34" s="26" t="n"/>
       <c r="E34" s="26" t="n"/>
       <c r="F34" s="26" t="n"/>
-      <c r="G34" s="27" t="n"/>
+      <c r="G34" s="26" t="n"/>
+      <c r="H34" s="26" t="n"/>
+      <c r="I34" s="26" t="n"/>
+      <c r="J34" s="27" t="n"/>
     </row>
     <row r="35" ht="15" customHeight="1" s="20">
       <c r="A35" s="28" t="n">
@@ -27214,7 +27337,10 @@
       <c r="D35" s="26" t="n"/>
       <c r="E35" s="26" t="n"/>
       <c r="F35" s="26" t="n"/>
-      <c r="G35" s="27" t="n"/>
+      <c r="G35" s="26" t="n"/>
+      <c r="H35" s="26" t="n"/>
+      <c r="I35" s="26" t="n"/>
+      <c r="J35" s="27" t="n"/>
     </row>
     <row r="36" ht="15" customHeight="1" s="20">
       <c r="A36" s="28" t="n">
@@ -27225,7 +27351,10 @@
       <c r="D36" s="26" t="n"/>
       <c r="E36" s="26" t="n"/>
       <c r="F36" s="26" t="n"/>
-      <c r="G36" s="27" t="n"/>
+      <c r="G36" s="26" t="n"/>
+      <c r="H36" s="26" t="n"/>
+      <c r="I36" s="26" t="n"/>
+      <c r="J36" s="27" t="n"/>
     </row>
     <row r="37" ht="15" customHeight="1" s="20">
       <c r="A37" s="28" t="n">
@@ -27236,7 +27365,10 @@
       <c r="D37" s="26" t="n"/>
       <c r="E37" s="26" t="n"/>
       <c r="F37" s="26" t="n"/>
-      <c r="G37" s="27" t="n"/>
+      <c r="G37" s="26" t="n"/>
+      <c r="H37" s="26" t="n"/>
+      <c r="I37" s="26" t="n"/>
+      <c r="J37" s="27" t="n"/>
     </row>
     <row r="38" ht="15" customHeight="1" s="20">
       <c r="A38" s="28" t="n">
@@ -27247,7 +27379,10 @@
       <c r="D38" s="26" t="n"/>
       <c r="E38" s="26" t="n"/>
       <c r="F38" s="26" t="n"/>
-      <c r="G38" s="27" t="n"/>
+      <c r="G38" s="26" t="n"/>
+      <c r="H38" s="26" t="n"/>
+      <c r="I38" s="26" t="n"/>
+      <c r="J38" s="27" t="n"/>
     </row>
     <row r="39" ht="15" customHeight="1" s="20">
       <c r="A39" s="28" t="n">
@@ -27258,7 +27393,10 @@
       <c r="D39" s="26" t="n"/>
       <c r="E39" s="26" t="n"/>
       <c r="F39" s="26" t="n"/>
-      <c r="G39" s="27" t="n"/>
+      <c r="G39" s="26" t="n"/>
+      <c r="H39" s="26" t="n"/>
+      <c r="I39" s="26" t="n"/>
+      <c r="J39" s="27" t="n"/>
     </row>
     <row r="40" ht="15" customHeight="1" s="20">
       <c r="A40" s="28" t="n">
@@ -27269,8 +27407,13 @@
       <c r="D40" s="26" t="n"/>
       <c r="E40" s="26" t="n"/>
       <c r="F40" s="26" t="n"/>
-      <c r="G40" s="27" t="n"/>
-    </row>
+      <c r="G40" s="26" t="n"/>
+      <c r="H40" s="26" t="n"/>
+      <c r="I40" s="26" t="n"/>
+      <c r="J40" s="27" t="n"/>
+    </row>
+    <row r="41"/>
+    <row r="42"/>
     <row r="43" ht="15" customHeight="1" s="20">
       <c r="A43" s="34" t="inlineStr">
         <is>
@@ -28207,7 +28350,7 @@
           <t>**Covid-19 cases ↓ this week.** Mono County reported 1 Covid-19 case, 0 flu cases, and 0 RSV cases for 10/5–10/11. Season-to-date since 9/7: 18 Covid-19, 1 flu, 1 RSV.</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="19" t="inlineStr">
         <is>
           <t>Mono County cases</t>
         </is>
@@ -28222,7 +28365,7 @@
           <t>**Covid-19 positivity ↓ 14%** (1 of 7 tests), down from 31% the prior week. All 11 flu tests and all 11 RSV tests were negative.</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="19" t="inlineStr">
         <is>
           <t>Test positivity</t>
         </is>
@@ -28237,7 +28380,7 @@
           <t>**2 flu patients, both influenza A**, neither a Mono County resident. No Covid-19 or RSV patients. Local wastewater sampling paused since 9/9.</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="19" t="inlineStr">
         <is>
           <t>Mammoth Hospital</t>
         </is>
@@ -28292,7 +28435,7 @@
           <t>**Fewer local cases this week.** Mono County reported 1 Covid-19 case (↓ from 6), 3 flu cases (↓ from 7), and 1 RSV case for 10/19–10/25. Season-to-date since 9/7: 25 Covid-19, 11 flu, 2 RSV.</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="19" t="inlineStr">
         <is>
           <t>Mono County cases</t>
         </is>
@@ -28307,7 +28450,7 @@
           <t>**Flu positivity ↓ 23%** (3 of 13 tests), down from 33% the prior week. Covid-19 ↓ 10% (1 of 10), down from 50%. RSV 8% (1 of 12).</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="19" t="inlineStr">
         <is>
           <t>Test positivity</t>
         </is>
@@ -28322,7 +28465,7 @@
           <t>**4 flu patients, mostly influenza A** (3 A, 1 B). 3 were Mono County residents; 2 of the 4 were vaccinated. 1 RSV patient (not a Mono County resident); no Covid-19 patients.</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="19" t="inlineStr">
         <is>
           <t>Mammoth Hospital</t>
         </is>
@@ -28337,7 +28480,7 @@
           <t>**Local sampling resumed 10/21.** SARS-CoV-2 detected at a level similar to early September. Influenza A, influenza B, and RSV not detected; the influenza A H1 subtype was detected at a low level. UC Davis trends return once more samples are collected.</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="19" t="inlineStr">
         <is>
           <t>Wastewater</t>
         </is>

</xml_diff>